<commit_message>
added comment dto files and comment mapper
</commit_message>
<xml_diff>
--- a/ipa_timeplan_sheungtsunglam.xlsx
+++ b/ipa_timeplan_sheungtsunglam.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myoffice.accenture.com/personal/masa_lam_accenture_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\masa.lam\0_ipa\equity-insight\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="434" documentId="8_{52ABB401-E745-4758-BDD8-91D4082E9887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7714048-88EF-4009-A91A-E71DD05EDD95}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9E329F-FD1F-48D6-8D76-91F0E2C20A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F000D33A-2255-403B-81DF-EEBC7025E60B}"/>
   </bookViews>
@@ -458,10 +458,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4125,7 +4121,9 @@
       <c r="AG35" s="8"/>
       <c r="AH35" s="8"/>
       <c r="AI35" s="8"/>
-      <c r="AJ35" s="8"/>
+      <c r="AJ35" s="15">
+        <v>1</v>
+      </c>
       <c r="AK35" s="8"/>
       <c r="AL35" s="8"/>
       <c r="AM35" s="8"/>
@@ -4314,13 +4312,27 @@
       <c r="AH37" s="8"/>
       <c r="AI37" s="8"/>
       <c r="AJ37" s="8"/>
-      <c r="AK37" s="8"/>
-      <c r="AL37" s="8"/>
-      <c r="AM37" s="8"/>
-      <c r="AN37" s="8"/>
-      <c r="AO37" s="8"/>
-      <c r="AP37" s="8"/>
-      <c r="AQ37" s="8"/>
+      <c r="AK37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AL37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AM37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AN37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AO37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AP37" s="15">
+        <v>1</v>
+      </c>
+      <c r="AQ37" s="15">
+        <v>1</v>
+      </c>
       <c r="AR37" s="8"/>
       <c r="AS37" s="8"/>
       <c r="AT37" s="8"/>

</xml_diff>